<commit_message>
Allineamento fogli di dettaglio, nuove cartelle gare e backup
- Prospetto.xlsx: sincronizzati i fogli di dettaglio col master (MIES proroga 07/10 + offerta presentata; Azienda Zero 5 lotti e ATI Getec 51%/Innova 49%; Lazio ATI Getec 70%/CS 30%); terminologia italianizzata (TBD->Da definire, ND->n.d.)
- Appalti: nuove cartelle per GVE fase 2 (con avviso TED 455567-2026), Comune di Roma, Policlinico di Milano, Ancona Torrette (con schede info)
- Aggiunte versioni/copie di lavorazione (Prospetto10/11, copie di backup)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Prospetto.xlsx
+++ b/Prospetto.xlsx
@@ -1865,7 +1865,7 @@
       </c>
       <c r="E9" s="100" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Da definire</t>
         </is>
       </c>
       <c r="F9" s="100" t="n"/>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="O9" s="100" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Da definire</t>
         </is>
       </c>
       <c r="P9" s="102" t="n"/>
@@ -1937,7 +1937,7 @@
       </c>
       <c r="E10" s="100" t="inlineStr">
         <is>
-          <t>TBD (max 1)</t>
+          <t>Da definire (max 1)</t>
         </is>
       </c>
       <c r="F10" s="100" t="n"/>
@@ -1973,7 +1973,7 @@
       </c>
       <c r="O10" s="100" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Da definire</t>
         </is>
       </c>
       <c r="P10" s="102" t="n"/>
@@ -2029,75 +2029,75 @@
       </c>
       <c r="C12" s="102" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="D12" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="E12" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="F12" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="G12" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H12" s="102" t="n"/>
       <c r="I12" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="J12" s="103" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="K12" s="103" t="n"/>
       <c r="L12" s="103" t="n"/>
       <c r="M12" s="101" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="N12" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="O12" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="P12" s="102" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="Q12" s="102" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="R12" s="101" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Da definire</t>
         </is>
       </c>
       <c r="S12" s="101" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Da definire</t>
         </is>
       </c>
       <c r="T12" s="101" t="n"/>
@@ -2136,14 +2136,14 @@
       </c>
       <c r="J13" s="103" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="K13" s="103" t="n"/>
       <c r="L13" s="103" t="n"/>
       <c r="M13" s="101" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="N13" s="100" t="inlineStr">
@@ -2158,12 +2158,12 @@
       </c>
       <c r="P13" s="102" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="Q13" s="102" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="R13" s="101" t="inlineStr">
@@ -2195,7 +2195,7 @@
       </c>
       <c r="C14" s="102" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="D14" s="100" t="n">
@@ -2209,7 +2209,7 @@
       </c>
       <c r="G14" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H14" s="102" t="n"/>
@@ -2220,14 +2220,14 @@
       </c>
       <c r="J14" s="103" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="K14" s="103" t="n"/>
       <c r="L14" s="103" t="n"/>
       <c r="M14" s="101" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="N14" s="100" t="inlineStr">
@@ -2237,17 +2237,17 @@
       </c>
       <c r="O14" s="100" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Da definire</t>
         </is>
       </c>
       <c r="P14" s="102" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="Q14" s="102" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="R14" s="101" t="inlineStr">
@@ -2315,78 +2315,78 @@
       </c>
       <c r="C16" s="102" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="D16" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="E16" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="F16" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="G16" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H16" s="102" t="n"/>
       <c r="I16" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="J16" s="103" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="K16" s="103" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="L16" s="103" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="M16" s="101" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="N16" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="O16" s="100" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Da definire</t>
         </is>
       </c>
       <c r="P16" s="102" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="Q16" s="102" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="R16" s="101" t="inlineStr">
         <is>
-          <t>TBD (probabile Getec/Innova/CS come fase 1)</t>
+          <t>Da definire (probabile Getec/Innova/CS come fase 1)</t>
         </is>
       </c>
       <c r="S16" s="101" t="inlineStr">
@@ -2409,73 +2409,73 @@
       </c>
       <c r="C17" s="102" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="D17" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="E17" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="F17" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="G17" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H17" s="102" t="n"/>
       <c r="I17" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="J17" s="103" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="K17" s="103" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="L17" s="103" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="M17" s="101" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="N17" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="O17" s="100" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Da definire</t>
         </is>
       </c>
       <c r="P17" s="102" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="Q17" s="102" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="R17" s="101" t="inlineStr">
@@ -2503,73 +2503,73 @@
       </c>
       <c r="C18" s="102" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="D18" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="E18" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="F18" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="G18" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H18" s="102" t="n"/>
       <c r="I18" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="J18" s="103" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="K18" s="103" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="L18" s="103" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="M18" s="101" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="N18" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="O18" s="100" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Da definire</t>
         </is>
       </c>
       <c r="P18" s="102" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="Q18" s="102" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="R18" s="101" t="inlineStr">
@@ -2597,73 +2597,73 @@
       </c>
       <c r="C19" s="102" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="D19" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="E19" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="F19" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="G19" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="H19" s="102" t="n"/>
       <c r="I19" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="J19" s="103" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="K19" s="103" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="L19" s="103" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="M19" s="101" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="N19" s="100" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="O19" s="100" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Da definire</t>
         </is>
       </c>
       <c r="P19" s="102" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="Q19" s="102" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="R19" s="101" t="inlineStr">
@@ -5016,7 +5016,7 @@
       </c>
       <c r="B3" s="136" t="inlineStr">
         <is>
-          <t>10 settembre 2026 — bando pubblicato</t>
+          <t>9 ottobre 2026 — offerta presentata (scadenza prorogata al 07/10)</t>
         </is>
       </c>
     </row>
@@ -5028,7 +5028,7 @@
       </c>
       <c r="B4" s="82" t="inlineStr">
         <is>
-          <t>🔴 BANDO PUBBLICATO — offerte 30/09/2026</t>
+          <t>✅ OFFERTA PRESENTATA da Certosa — offerte prorogate al 07/10/2026 (chiuse)</t>
         </is>
       </c>
     </row>
@@ -5210,7 +5210,7 @@
       </c>
       <c r="B22" s="82" t="inlineStr">
         <is>
-          <t>30/09/2026 ore 16:00</t>
+          <t>07/10/2026 (prorogata) — offerta Certosa presentata</t>
         </is>
       </c>
     </row>
@@ -5222,7 +5222,7 @@
       </c>
       <c r="B23" s="82" t="inlineStr">
         <is>
-          <t>02/10/2026 ore 15:00 — INVERSIONE PROCEDIMENTALE</t>
+          <t>da ridefinire (post proroga) — inversione procedimentale</t>
         </is>
       </c>
     </row>
@@ -6587,7 +6587,7 @@
       </c>
       <c r="B81" s="136" t="inlineStr">
         <is>
-          <t>Precedente configurazione tracciata: GETEC 80% + Certosa Servizi 20%. Da RICONFERMARE per Ed. 4 in funzione del/dei lotti scelti.</t>
+          <t>ATI CONFERMATA: GETEC 70% (mandataria) + Certosa Servizi 30% (mandante). Getec copre anche i requisiti di Certosa Servizi.</t>
         </is>
       </c>
     </row>
@@ -7673,7 +7673,7 @@
       </c>
       <c r="E58" s="22" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Da definire</t>
         </is>
       </c>
       <c r="F58" s="24" t="inlineStr">
@@ -7696,7 +7696,7 @@
       </c>
       <c r="E59" s="22" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Da definire</t>
         </is>
       </c>
       <c r="F59" s="24" t="inlineStr">
@@ -7716,12 +7716,12 @@
       </c>
       <c r="D60" s="23" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
       <c r="E60" s="23" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Da definire</t>
         </is>
       </c>
       <c r="F60" s="24" t="inlineStr">
@@ -11110,7 +11110,7 @@
       </c>
       <c r="B12" s="136" t="inlineStr">
         <is>
-          <t>ND</t>
+          <t>n.d.</t>
         </is>
       </c>
     </row>
@@ -11260,7 +11260,7 @@
       </c>
       <c r="B6" s="136" t="inlineStr">
         <is>
-          <t>AGGIUDICATA — Con ricorsi pendenti al TAR</t>
+          <t>AGGIUDICATA (DDG 658 del 16/09/2025) — ricorsi pendenti al TAR</t>
         </is>
       </c>
     </row>
@@ -11392,8 +11392,10 @@
           <t>Lotti</t>
         </is>
       </c>
-      <c r="B20" s="136" t="n">
-        <v>6</v>
+      <c r="B20" s="136" t="inlineStr">
+        <is>
+          <t>5 per Certosa (bando 6 lotti; Lotto 6 ULSS 9 → Teckal, fuori perimetro)</t>
+        </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="118">
@@ -11490,7 +11492,7 @@
       </c>
       <c r="B31" s="136" t="inlineStr">
         <is>
-          <t>GETEC (80%)</t>
+          <t>GETEC (51%)</t>
         </is>
       </c>
     </row>
@@ -11502,7 +11504,7 @@
       </c>
       <c r="B32" s="136" t="inlineStr">
         <is>
-          <t>Certosa Servizi (20%)</t>
+          <t>Cons. Innova (49%): Certosa Servizi 25% + Innova 24%</t>
         </is>
       </c>
     </row>

</xml_diff>